<commit_message>
- Introduced runState.ts to manage state persistence across test runs, allowing tests to share values and handle blocking steps effectively. - fixed blocking scenarios for each product -DNY
</commit_message>
<xml_diff>
--- a/PPP/PPP_Schedule_Import.xlsx
+++ b/PPP/PPP_Schedule_Import.xlsx
@@ -1461,8 +1461,10 @@
       <c r="CG2" t="s">
         <v>139</v>
       </c>
-      <c r="CH2" t="s">
-        <v>109</v>
+      <c r="CH2" t="inlineStr">
+        <is>
+          <t>Survey Completed</t>
+        </is>
       </c>
       <c r="CI2" t="s">
         <v>127</v>

</xml_diff>